<commit_message>
Update linkage workbook, footer
</commit_message>
<xml_diff>
--- a/assets/resources/docs/Linkage_Request_Planning_Workbook_final.xlsx
+++ b/assets/resources/docs/Linkage_Request_Planning_Workbook_final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shull/Documents/2026 NCI Data Linkage/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mitre.sharepoint.com/sites/ncilegalethicsgovernanceframework/Shared Documents/Task 3 - Refine Legal and Ethics Gov Framework/Implementation Materials/Linkage Workbook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC09597D-2102-0143-9225-1820088DC597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{FC09597D-2102-0143-9225-1820088DC597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF5B1709-0480-FF46-9A46-0FCB33BD07F5}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19200" tabRatio="682" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="520" windowWidth="26240" windowHeight="16440" tabRatio="682" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ABOUT" sheetId="10" r:id="rId1"/>
@@ -52,9 +52,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="292">
   <si>
-    <t>Data Linkage Planning Workbook</t>
-  </si>
-  <si>
     <t>PURPOSE</t>
   </si>
   <si>
@@ -993,6 +990,9 @@
     <t>The views, opinions and/or findings contained in this report are those of The MITRE Corporation and should not be construed as an official government position, policy, or decision, unless designated by other documentation. This technical data report was produced for the U.S. Government under Contract Number 75FCMC23D0004, and is subject to Federal Acquisition Regulation Clause 52.227-14, Rights in Data-General. No other use other than that granted to the U.S. Government, or to those acting on behalf of the U.S. Government under that Clause is authorized without the express written permission of The MITRE Corporation. 
 For further information, please contact The MITRE Corporation, Contracts Management Office, 7515 Colshire Drive, McLean, VA 22102-7539, (703) 983-6000. 
 © 2026 The MITRE Corporation.</t>
+  </si>
+  <si>
+    <t>Linkage Request Planning Workbook</t>
   </si>
 </sst>
 </file>
@@ -1460,6 +1460,36 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1471,36 +1501,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1536,9 +1536,6 @@
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -1552,6 +1549,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1850,117 +1850,109 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" s="4" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="43" t="s">
+      <c r="B1" s="39" t="s">
+        <v>291</v>
+      </c>
+      <c r="C1" s="39"/>
+      <c r="E1" s="5"/>
+    </row>
+    <row r="2" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="E1" s="5"/>
-    </row>
-    <row r="2" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="41" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="42"/>
+      <c r="C2" s="38"/>
     </row>
     <row r="3" spans="2:7" s="2" customFormat="1" ht="118" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="44" t="s">
-        <v>288</v>
-      </c>
-      <c r="C3" s="45"/>
+      <c r="B3" s="40" t="s">
+        <v>287</v>
+      </c>
+      <c r="C3" s="41"/>
     </row>
     <row r="4" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="C4" s="42"/>
+      <c r="B4" s="37" t="s">
+        <v>122</v>
+      </c>
+      <c r="C4" s="38"/>
     </row>
     <row r="5" spans="2:7" ht="122" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="44" t="s">
-        <v>158</v>
-      </c>
-      <c r="C5" s="45"/>
+      <c r="B5" s="40" t="s">
+        <v>157</v>
+      </c>
+      <c r="C5" s="41"/>
     </row>
     <row r="6" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C6" s="10"/>
     </row>
     <row r="7" spans="2:7" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="36" t="s">
-        <v>159</v>
-      </c>
-      <c r="C7" s="37"/>
+      <c r="B7" s="32" t="s">
+        <v>158</v>
+      </c>
+      <c r="C7" s="33"/>
     </row>
     <row r="8" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="39" t="s">
+      <c r="B8" s="35" t="s">
+        <v>289</v>
+      </c>
+      <c r="C8" s="36"/>
+    </row>
+    <row r="9" spans="2:7" ht="89" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="34" t="s">
         <v>290</v>
       </c>
-      <c r="C8" s="40"/>
-    </row>
-    <row r="9" spans="2:7" ht="89" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="38" t="s">
-        <v>291</v>
-      </c>
-      <c r="C9" s="38"/>
+      <c r="C9" s="34"/>
       <c r="G9" s="4"/>
     </row>
     <row r="10" spans="2:7" s="4" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="33" t="s">
-        <v>289</v>
-      </c>
-      <c r="C10" s="33"/>
+      <c r="B10" s="43" t="s">
+        <v>288</v>
+      </c>
+      <c r="C10" s="43"/>
     </row>
     <row r="11" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="34"/>
-      <c r="C11" s="34"/>
+      <c r="B11" s="44"/>
+      <c r="C11" s="44"/>
     </row>
     <row r="12" spans="2:7" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
     </row>
     <row r="13" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
+      <c r="B13" s="45"/>
+      <c r="C13" s="45"/>
     </row>
     <row r="14" spans="2:7" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="34"/>
-      <c r="C14" s="34"/>
+      <c r="B14" s="44"/>
+      <c r="C14" s="44"/>
     </row>
     <row r="15" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="35"/>
-      <c r="C15" s="35"/>
+      <c r="B15" s="45"/>
+      <c r="C15" s="45"/>
     </row>
     <row r="16" spans="2:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="34"/>
-      <c r="C16" s="34"/>
+      <c r="B16" s="44"/>
+      <c r="C16" s="44"/>
     </row>
     <row r="17" spans="2:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="35"/>
-      <c r="C17" s="35"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="45"/>
     </row>
     <row r="18" spans="2:3" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="34"/>
-      <c r="C18" s="34"/>
+      <c r="B18" s="44"/>
+      <c r="C18" s="44"/>
     </row>
     <row r="19" spans="2:3" ht="9.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
     </row>
     <row r="20" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="32"/>
-      <c r="C20" s="32"/>
+      <c r="B20" s="42"/>
+      <c r="C20" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B5:C5"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
@@ -1970,6 +1962,14 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B5:C5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1991,80 +1991,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="43" t="s">
-        <v>116</v>
-      </c>
-      <c r="C1" s="43"/>
+      <c r="B1" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="39"/>
     </row>
     <row r="2" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C2" s="14"/>
     </row>
     <row r="3" spans="2:3" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="36" t="s">
-        <v>282</v>
-      </c>
-      <c r="C3" s="37"/>
+      <c r="B3" s="32" t="s">
+        <v>281</v>
+      </c>
+      <c r="C3" s="33"/>
     </row>
     <row r="4" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="47" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C4" s="48"/>
     </row>
     <row r="5" spans="2:3" s="4" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="49" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C5" s="50"/>
     </row>
     <row r="6" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="47" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C6" s="48"/>
     </row>
     <row r="7" spans="2:3" ht="47" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="51" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C7" s="52"/>
     </row>
     <row r="8" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="47" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C8" s="48"/>
     </row>
     <row r="9" spans="2:3" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="51" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C9" s="52"/>
     </row>
     <row r="10" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="47" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C10" s="48"/>
     </row>
     <row r="11" spans="2:3" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="51" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C11" s="52"/>
     </row>
     <row r="12" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="47" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C12" s="48"/>
     </row>
     <row r="13" spans="2:3" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="53" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C13" s="54"/>
     </row>
@@ -2074,64 +2074,64 @@
     </row>
     <row r="15" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="55" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C15" s="56"/>
     </row>
     <row r="16" spans="2:3" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="17" spans="2:3" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="2:3" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="19" spans="2:3" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="2:3" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="18" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="21" spans="2:3" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="22" spans="2:3" s="7" customFormat="1" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="20" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="23" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -2140,128 +2140,128 @@
     </row>
     <row r="24" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="55" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C24" s="56"/>
     </row>
     <row r="25" spans="2:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="26" spans="2:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="21" t="s">
+        <v>168</v>
+      </c>
+      <c r="C26" s="15" t="s">
         <v>169</v>
-      </c>
-      <c r="C26" s="15" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="21" t="s">
+        <v>171</v>
+      </c>
+      <c r="C27" s="23" t="s">
         <v>172</v>
-      </c>
-      <c r="C27" s="23" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="28" spans="2:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" spans="2:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="21" t="s">
+        <v>173</v>
+      </c>
+      <c r="C29" s="15" t="s">
         <v>174</v>
-      </c>
-      <c r="C29" s="15" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="15" t="s">
         <v>5</v>
-      </c>
-      <c r="C30" s="15" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="21" t="s">
+        <v>175</v>
+      </c>
+      <c r="C31" s="15" t="s">
         <v>176</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="32" spans="2:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="21" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="33" spans="2:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="21" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="34" spans="2:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C34" s="15" t="s">
         <v>12</v>
-      </c>
-      <c r="C34" s="15" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="35" spans="2:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="21" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="36" spans="2:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B36" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" s="15" t="s">
         <v>9</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="37" spans="2:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="38" spans="2:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="21" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="39" spans="2:5" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="C39" s="16" t="s">
         <v>3</v>
-      </c>
-      <c r="C39" s="16" t="s">
-        <v>4</v>
       </c>
       <c r="E39" s="1"/>
     </row>
@@ -2319,297 +2319,313 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="61" t="s">
-        <v>91</v>
-      </c>
-      <c r="C1" s="61"/>
+      <c r="B1" s="60" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" s="60"/>
     </row>
     <row r="2" spans="2:3" ht="93" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="62" t="s">
-        <v>181</v>
-      </c>
-      <c r="C2" s="63"/>
+      <c r="B2" s="61" t="s">
+        <v>180</v>
+      </c>
+      <c r="C2" s="62"/>
     </row>
     <row r="3" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
     </row>
     <row r="4" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="59" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="59"/>
+      <c r="B4" s="58" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="58"/>
     </row>
     <row r="5" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="31" t="s">
-        <v>20</v>
-      </c>
     </row>
     <row r="6" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="58" t="s">
-        <v>127</v>
-      </c>
-      <c r="C6" s="58"/>
+      <c r="B6" s="63" t="s">
+        <v>126</v>
+      </c>
+      <c r="C6" s="63"/>
     </row>
     <row r="7" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
     </row>
     <row r="8" spans="2:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="59" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="59"/>
+      <c r="B8" s="58" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="58"/>
     </row>
     <row r="9" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C9" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="57" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C10" s="57"/>
     </row>
     <row r="11" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="12" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="59" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="59"/>
+      <c r="B12" s="58" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="58"/>
     </row>
     <row r="13" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="24" t="s">
+        <v>181</v>
+      </c>
+      <c r="C13" s="26" t="s">
         <v>182</v>
       </c>
-      <c r="C13" s="26" t="s">
+    </row>
+    <row r="14" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="59" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="14" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="60" t="s">
-        <v>184</v>
-      </c>
-      <c r="C14" s="60"/>
+      <c r="C14" s="59"/>
     </row>
     <row r="15" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="16" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="59" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" s="59"/>
+      <c r="B16" s="58" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="58"/>
     </row>
     <row r="17" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="24" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="57" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C18" s="57"/>
     </row>
     <row r="19" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="20" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="59" t="s">
-        <v>93</v>
-      </c>
-      <c r="C20" s="59"/>
+      <c r="B20" s="58" t="s">
+        <v>92</v>
+      </c>
+      <c r="C20" s="58"/>
     </row>
     <row r="21" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="26" t="s">
+    </row>
+    <row r="22" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="59" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="22" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="60" t="s">
-        <v>28</v>
-      </c>
-      <c r="C22" s="60"/>
+      <c r="C22" s="59"/>
     </row>
     <row r="23" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="27" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="57" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C24" s="57"/>
     </row>
     <row r="25" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="24" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C25" s="26" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="26" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="57" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C26" s="57"/>
     </row>
     <row r="27" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="24" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="28" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="57" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C28" s="57"/>
     </row>
     <row r="29" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C29" s="26" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="57" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C30" s="57"/>
     </row>
     <row r="31" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="32" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="59" t="s">
-        <v>119</v>
-      </c>
-      <c r="C32" s="59"/>
+      <c r="B32" s="58" t="s">
+        <v>118</v>
+      </c>
+      <c r="C32" s="58"/>
     </row>
     <row r="33" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" s="26" t="s">
         <v>33</v>
-      </c>
-      <c r="C33" s="26" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="34" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="57" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C34" s="57"/>
     </row>
     <row r="35" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="24" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C35" s="26" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="36" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B36" s="57" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C36" s="57"/>
     </row>
     <row r="37" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="38" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="59" t="s">
-        <v>94</v>
-      </c>
-      <c r="C38" s="59"/>
+      <c r="B38" s="58" t="s">
+        <v>93</v>
+      </c>
+      <c r="C38" s="58"/>
     </row>
     <row r="39" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="24" t="s">
+        <v>193</v>
+      </c>
+      <c r="C39" s="26" t="s">
         <v>194</v>
-      </c>
-      <c r="C39" s="26" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="40" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="57" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C40" s="57"/>
     </row>
     <row r="41" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="42" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="59" t="s">
-        <v>95</v>
-      </c>
-      <c r="C42" s="59"/>
+      <c r="B42" s="58" t="s">
+        <v>94</v>
+      </c>
+      <c r="C42" s="58"/>
     </row>
     <row r="43" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B43" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C43" s="26" t="s">
         <v>36</v>
-      </c>
-      <c r="C43" s="26" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="44" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B44" s="57" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C44" s="57"/>
     </row>
     <row r="46" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B46" s="59" t="s">
-        <v>96</v>
-      </c>
-      <c r="C46" s="59"/>
+      <c r="B46" s="58" t="s">
+        <v>95</v>
+      </c>
+      <c r="C46" s="58"/>
     </row>
     <row r="47" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B47" s="24" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C47" s="26" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="48" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B48" s="57" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C48" s="57"/>
     </row>
     <row r="49" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B49" s="24" t="s">
+        <v>199</v>
+      </c>
+      <c r="C49" s="26" t="s">
         <v>200</v>
-      </c>
-      <c r="C49" s="26" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="50" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="57" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C50" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B10:C10"/>
     <mergeCell ref="B44:C44"/>
     <mergeCell ref="B48:C48"/>
     <mergeCell ref="B50:C50"/>
@@ -2620,22 +2636,6 @@
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B14:C14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2657,70 +2657,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="61" t="s">
-        <v>118</v>
-      </c>
-      <c r="C1" s="61"/>
+      <c r="B1" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="C1" s="60"/>
     </row>
     <row r="2" spans="2:3" ht="77" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="64" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C2" s="65"/>
     </row>
     <row r="3" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="66" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C4" s="66"/>
     </row>
     <row r="5" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="24" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="57" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C6" s="57"/>
     </row>
     <row r="7" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="8" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="66" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C8" s="66"/>
     </row>
     <row r="9" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="24" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="57" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C10" s="57"/>
     </row>
     <row r="11" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="24" t="s">
+        <v>207</v>
+      </c>
+      <c r="C11" s="26" t="s">
         <v>208</v>
-      </c>
-      <c r="C11" s="26" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="57" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C12" s="57"/>
     </row>
@@ -2754,126 +2754,126 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="61" t="s">
-        <v>97</v>
-      </c>
-      <c r="C1" s="61"/>
+      <c r="B1" s="60" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="60"/>
     </row>
     <row r="2" spans="2:3" ht="108" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="64" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C2" s="65"/>
     </row>
     <row r="3" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="66" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C4" s="66"/>
     </row>
     <row r="5" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="24" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="57" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C6" s="57"/>
     </row>
     <row r="7" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="24" t="s">
+        <v>211</v>
+      </c>
+      <c r="C7" s="26" t="s">
         <v>212</v>
-      </c>
-      <c r="C7" s="26" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="57" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C8" s="57"/>
     </row>
     <row r="9" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="26" t="s">
         <v>41</v>
-      </c>
-      <c r="C9" s="26" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="57" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C10" s="57"/>
     </row>
     <row r="11" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="57" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C12" s="57"/>
     </row>
     <row r="13" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="14" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="66" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C14" s="66"/>
     </row>
     <row r="15" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="24" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="57" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C16" s="57"/>
     </row>
     <row r="17" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="C17" s="26" t="s">
         <v>216</v>
-      </c>
-      <c r="C17" s="26" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="57" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C18" s="57"/>
     </row>
     <row r="19" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" s="26" t="s">
         <v>47</v>
-      </c>
-      <c r="C19" s="26" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="57" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C20" s="57"/>
     </row>
@@ -2911,142 +2911,142 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="34.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="61" t="s">
-        <v>98</v>
-      </c>
-      <c r="C1" s="61"/>
+      <c r="B1" s="60" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1" s="60"/>
     </row>
     <row r="2" spans="2:3" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="53" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C2" s="54"/>
     </row>
     <row r="3" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="66" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C4" s="66"/>
     </row>
     <row r="5" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="28" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="57" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C6" s="57"/>
     </row>
     <row r="7" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" s="26" t="s">
         <v>51</v>
-      </c>
-      <c r="C7" s="26" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="57" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C8" s="57"/>
     </row>
     <row r="9" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="57" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C10" s="57"/>
     </row>
     <row r="11" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="12" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="66" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C12" s="66"/>
     </row>
     <row r="13" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="24" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="57" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C14" s="57"/>
     </row>
     <row r="15" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="30" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="16" spans="2:3" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="57" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C16" s="57"/>
     </row>
     <row r="17" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="24" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="57" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C18" s="57"/>
     </row>
     <row r="19" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="24" t="s">
+        <v>223</v>
+      </c>
+      <c r="C19" s="26" t="s">
         <v>224</v>
-      </c>
-      <c r="C19" s="26" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="57" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C20" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B12:C12"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B12:C12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -3068,182 +3068,182 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" s="6" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="61" t="s">
-        <v>58</v>
-      </c>
-      <c r="C1" s="61"/>
+      <c r="B1" s="60" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="60"/>
     </row>
     <row r="2" spans="2:3" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="62" t="s">
-        <v>231</v>
-      </c>
-      <c r="C2" s="63"/>
+      <c r="B2" s="61" t="s">
+        <v>230</v>
+      </c>
+      <c r="C2" s="62"/>
     </row>
     <row r="3" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="2:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="66" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C4" s="66"/>
     </row>
     <row r="5" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="24" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="57" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C6" s="57"/>
     </row>
     <row r="7" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="24" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="57" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C8" s="57"/>
     </row>
     <row r="9" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="24" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="57" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C10" s="57"/>
     </row>
     <row r="11" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="24" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="57" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C12" s="57"/>
     </row>
     <row r="13" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="24" t="s">
+        <v>241</v>
+      </c>
+      <c r="C13" s="26" t="s">
         <v>242</v>
-      </c>
-      <c r="C13" s="26" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="14" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="57" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C14" s="57"/>
     </row>
     <row r="15" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="26" t="s">
         <v>60</v>
-      </c>
-      <c r="C15" s="26" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="16" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="57" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C16" s="57"/>
     </row>
     <row r="17" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="24" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="57" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C18" s="57"/>
     </row>
     <row r="19" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="20" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="66" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C20" s="66"/>
     </row>
     <row r="21" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="24" t="s">
+        <v>245</v>
+      </c>
+      <c r="C21" s="26" t="s">
         <v>246</v>
-      </c>
-      <c r="C21" s="26" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="22" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="57" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C22" s="57"/>
     </row>
     <row r="23" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="24" t="s">
+        <v>248</v>
+      </c>
+      <c r="C23" s="26" t="s">
         <v>249</v>
-      </c>
-      <c r="C23" s="26" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="57" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C24" s="57"/>
     </row>
     <row r="25" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="24" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C25" s="26" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="26" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="57" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C26" s="57"/>
     </row>
     <row r="27" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="24" t="s">
+        <v>252</v>
+      </c>
+      <c r="C27" s="26" t="s">
         <v>253</v>
-      </c>
-      <c r="C27" s="26" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="28" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="57" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C28" s="57"/>
     </row>
@@ -3285,203 +3285,203 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="61" t="s">
-        <v>99</v>
-      </c>
-      <c r="C1" s="61"/>
+      <c r="B1" s="60" t="s">
+        <v>98</v>
+      </c>
+      <c r="C1" s="60"/>
     </row>
     <row r="2" spans="2:3" ht="88" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="62" t="s">
-        <v>255</v>
-      </c>
-      <c r="C2" s="63"/>
+      <c r="B2" s="61" t="s">
+        <v>254</v>
+      </c>
+      <c r="C2" s="62"/>
     </row>
     <row r="3" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="66" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C4" s="66"/>
     </row>
     <row r="5" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="24" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="57" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C6" s="57"/>
     </row>
     <row r="7" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="24" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="53" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="57" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C8" s="57"/>
     </row>
     <row r="9" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="24" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="57" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C10" s="57"/>
     </row>
     <row r="11" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="59" t="s">
         <v>67</v>
       </c>
-      <c r="C11" s="26" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="12" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="60" t="s">
-        <v>68</v>
-      </c>
-      <c r="C12" s="60"/>
+      <c r="C12" s="59"/>
     </row>
     <row r="13" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="14" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="66" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C14" s="66"/>
     </row>
     <row r="15" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="24" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="16" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="57" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C16" s="57"/>
     </row>
     <row r="17" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="24" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="57" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C18" s="57"/>
     </row>
     <row r="19" spans="2:3" ht="23" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="20" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="66" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C20" s="66"/>
     </row>
     <row r="21" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="24" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="22" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="57" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C22" s="57"/>
     </row>
     <row r="23" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="C23" s="26" t="s">
         <v>73</v>
-      </c>
-      <c r="C23" s="26" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="57" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C24" s="57"/>
     </row>
     <row r="25" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="26" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="66" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C26" s="66"/>
     </row>
     <row r="27" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="28" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="57" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C28" s="57"/>
     </row>
     <row r="29" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="24" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C29" s="26" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="57" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C30" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B8:C8"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B22:C22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -3503,165 +3503,160 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="61" t="s">
-        <v>100</v>
-      </c>
-      <c r="C1" s="61"/>
+      <c r="B1" s="60" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1" s="60"/>
     </row>
     <row r="2" spans="2:3" ht="76" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="62" t="s">
-        <v>133</v>
-      </c>
-      <c r="C2" s="63"/>
+      <c r="B2" s="61" t="s">
+        <v>132</v>
+      </c>
+      <c r="C2" s="62"/>
     </row>
     <row r="3" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="66" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C4" s="66"/>
     </row>
     <row r="5" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="24" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="57" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C6" s="57"/>
     </row>
     <row r="7" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="24" t="s">
+        <v>264</v>
+      </c>
+      <c r="C7" s="26" t="s">
         <v>265</v>
-      </c>
-      <c r="C7" s="26" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="57" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C8" s="57"/>
     </row>
     <row r="9" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="24" t="s">
+        <v>137</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="59" t="s">
         <v>138</v>
       </c>
-      <c r="C9" s="26" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="10" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="60" t="s">
-        <v>139</v>
-      </c>
-      <c r="C10" s="60"/>
+      <c r="C10" s="59"/>
     </row>
     <row r="11" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="24" t="s">
+        <v>266</v>
+      </c>
+      <c r="C11" s="26" t="s">
         <v>267</v>
-      </c>
-      <c r="C11" s="26" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="57" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C12" s="57"/>
     </row>
     <row r="13" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="14" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="66" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C14" s="66"/>
     </row>
     <row r="15" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="24" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="2:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="57" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C16" s="57"/>
     </row>
     <row r="17" spans="2:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="24" t="s">
+        <v>269</v>
+      </c>
+      <c r="C17" s="26" t="s">
         <v>270</v>
-      </c>
-      <c r="C17" s="26" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="57" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C18" s="57"/>
     </row>
     <row r="19" spans="2:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="24" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="20" spans="2:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="67" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C20" s="67"/>
     </row>
     <row r="21" spans="2:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="24" t="s">
+        <v>272</v>
+      </c>
+      <c r="C21" s="26" t="s">
         <v>273</v>
-      </c>
-      <c r="C21" s="26" t="s">
-        <v>274</v>
       </c>
       <c r="E21" s="17"/>
     </row>
     <row r="22" spans="2:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="57" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C22" s="57"/>
     </row>
     <row r="23" spans="2:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="24" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="57" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C24" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B24:C24"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -3670,6 +3665,11 @@
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B24:C24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -3677,6 +3677,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="b5a44311-ed64-4a72-909f-c9dc6973bde2" xsi:nil="true"/>
@@ -3686,15 +3695,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3905,26 +3905,26 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF022A8B-3988-495E-B2B1-F59BF51B69DB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC7CE11F-0C8B-4F26-AD06-9E1EB8A5CF44}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="b5a44311-ed64-4a72-909f-c9dc6973bde2"/>
-    <ds:schemaRef ds:uri="1dd0de65-4588-429c-bed4-0bd2be557c9b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC7CE11F-0C8B-4F26-AD06-9E1EB8A5CF44}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF022A8B-3988-495E-B2B1-F59BF51B69DB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="1dd0de65-4588-429c-bed4-0bd2be557c9b"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b5a44311-ed64-4a72-909f-c9dc6973bde2"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>